<commit_message>
updates and backup before merging
</commit_message>
<xml_diff>
--- a/Results/1_preprocessing/iML1515_UES_intercept_screen.xlsx
+++ b/Results/1_preprocessing/iML1515_UES_intercept_screen.xlsx
@@ -402,7 +402,7 @@
         <v>0.7</v>
       </c>
       <c r="C2">
-        <v>0.1316488940627486</v>
+        <v>0.2269948405835983</v>
       </c>
       <c r="D2">
         <v>0</v>
@@ -416,7 +416,7 @@
         <v>0.7</v>
       </c>
       <c r="C3">
-        <v>-0.1068473418759518</v>
+        <v>0.1675827929333596</v>
       </c>
       <c r="D3">
         <v>1</v>
@@ -430,7 +430,7 @@
         <v>0.7</v>
       </c>
       <c r="C4">
-        <v>-0.3213049502479167</v>
+        <v>-0.3369107113573124</v>
       </c>
       <c r="D4">
         <v>2</v>
@@ -444,7 +444,7 @@
         <v>0.9149149521563553</v>
       </c>
       <c r="C5">
-        <v>0.05280826199388263</v>
+        <v>0.5992379925671577</v>
       </c>
       <c r="D5">
         <v>0</v>
@@ -458,7 +458,7 @@
         <v>0.9149149521563553</v>
       </c>
       <c r="C6">
-        <v>-0.4039099554791698</v>
+        <v>0.286614769681655</v>
       </c>
       <c r="D6">
         <v>1</v>
@@ -472,7 +472,7 @@
         <v>0.9149149521563553</v>
       </c>
       <c r="C7">
-        <v>0.4449768321185183</v>
+        <v>0.3742914051115787</v>
       </c>
       <c r="D7">
         <v>2</v>
@@ -486,7 +486,7 @@
         <v>1.129829904312711</v>
       </c>
       <c r="C8">
-        <v>-0.08523757230271485</v>
+        <v>-0.09269447259562098</v>
       </c>
       <c r="D8">
         <v>0</v>
@@ -500,7 +500,7 @@
         <v>1.129829904312711</v>
       </c>
       <c r="C9">
-        <v>0.2083778506327755</v>
+        <v>0.4365318651580543</v>
       </c>
       <c r="D9">
         <v>1</v>
@@ -514,7 +514,7 @@
         <v>1.129829904312711</v>
       </c>
       <c r="C10">
-        <v>-0.1310912746065364</v>
+        <v>-0.5821467758974715</v>
       </c>
       <c r="D10">
         <v>2</v>
@@ -528,7 +528,7 @@
         <v>1.344744856469066</v>
       </c>
       <c r="C11">
-        <v>-0.2916755379406467</v>
+        <v>0.4188445278721831</v>
       </c>
       <c r="D11">
         <v>0</v>
@@ -542,7 +542,7 @@
         <v>1.344744856469066</v>
       </c>
       <c r="C12">
-        <v>0.1503518084160289</v>
+        <v>0.4689069165208387</v>
       </c>
       <c r="D12">
         <v>1</v>
@@ -556,7 +556,7 @@
         <v>1.344744856469066</v>
       </c>
       <c r="C13">
-        <v>0.263910475876477</v>
+        <v>-0.2144279029009213</v>
       </c>
       <c r="D13">
         <v>2</v>

</xml_diff>